<commit_message>
chore(auto): save work in "\354\275\225\354\247\221 (1 file(s), 2026-09-11 10:49)
</commit_message>
<xml_diff>
--- a/콕집/KOKJIP_Signal_Dataset_v0.1_HumanReview.xlsx
+++ b/콕집/KOKJIP_Signal_Dataset_v0.1_HumanReview.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5134d5ca37da44c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signal Dataset" sheetId="2" r:id="R6041f492e00840c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="3" r:id="R5d7d4375fb8e4bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Review" sheetId="4" r:id="R8f6949d81c704c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R49106f5503d04890"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signal Dataset" sheetId="2" r:id="R2887ff91fd574893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="3" r:id="Rf5401a04faf547c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Review" sheetId="4" r:id="R674c2ebd44c9471f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4179,7 +4179,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35a39f51ee734688"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff3b368555644e4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4349,7 +4349,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra06a0be8a3134168"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3d611eff197458f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4497,16 +4497,16 @@
           <x:t xml:space="preserve">복습 우선순위가 높은 핵심 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I2" s="11" t="str"/>
+      <x:c r="I2" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J2" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K2" s="11" t="str">
-        <x:v>강조</x:v>
-      </x:c>
-      <x:c r="L2" s="11" t="n">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K2" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L2" s="11" t="str"/>
       <x:c r="M2" s="11" t="str"/>
       <x:c r="N2" s="11" t="str"/>
       <x:c r="P2" s="11" t="inlineStr">
@@ -4559,16 +4559,16 @@
           <x:t xml:space="preserve">구현 시 재사용 가능한 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I3" s="11" t="str"/>
+      <x:c r="I3" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J3" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K3" s="11" t="str">
-        <x:v>강조</x:v>
-      </x:c>
-      <x:c r="L3" s="11" t="n">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K3" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L3" s="11" t="str"/>
       <x:c r="M3" s="11" t="str"/>
       <x:c r="N3" s="11" t="str"/>
       <x:c r="P3" s="11" t="inlineStr">
@@ -4621,16 +4621,16 @@
           <x:t xml:space="preserve">설계 품질 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I4" s="11" t="str"/>
+      <x:c r="I4" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J4" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K4" s="11" t="str">
-        <x:v>강조</x:v>
-      </x:c>
-      <x:c r="L4" s="11" t="n">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K4" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L4" s="11" t="str"/>
       <x:c r="M4" s="11" t="str"/>
       <x:c r="N4" s="11" t="str"/>
       <x:c r="P4" s="11" t="inlineStr">
@@ -4683,16 +4683,16 @@
           <x:t xml:space="preserve">필수 행동으로 제시</x:t>
         </x:is>
       </x:c>
-      <x:c r="I5" s="11" t="str"/>
+      <x:c r="I5" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J5" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K5" s="11" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="L5" s="11" t="n">
+        <x:v>MUST</x:v>
+      </x:c>
+      <x:c r="K5" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L5" s="11" t="str"/>
       <x:c r="M5" s="11" t="str"/>
       <x:c r="N5" s="11" t="str"/>
       <x:c r="P5" s="11" t="inlineStr">
@@ -4745,16 +4745,16 @@
           <x:t xml:space="preserve">MVP 판단 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I6" s="11" t="str"/>
+      <x:c r="I6" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J6" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K6" s="11" t="str">
-        <x:v>필수</x:v>
-      </x:c>
-      <x:c r="L6" s="11" t="n">
+        <x:v>MUST</x:v>
+      </x:c>
+      <x:c r="K6" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L6" s="11" t="str"/>
       <x:c r="M6" s="11" t="str"/>
       <x:c r="N6" s="11" t="str"/>
       <x:c r="P6" s="11" t="inlineStr">
@@ -4807,12 +4807,12 @@
           <x:t xml:space="preserve">실행 가능성 판단 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I7" s="11" t="str"/>
-      <x:c r="J7" s="11" t="str">
+      <x:c r="I7" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K7" s="11"/>
-      <x:c r="L7" s="11"/>
+      <x:c r="J7" s="11" t="str"/>
+      <x:c r="K7" s="11" t="str"/>
+      <x:c r="L7" s="11" t="str"/>
       <x:c r="M7" s="11" t="str"/>
       <x:c r="N7" s="11" t="str"/>
       <x:c r="P7" s="11" t="inlineStr">
@@ -4865,12 +4865,12 @@
           <x:t xml:space="preserve">프로젝트 단계 전환 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I8" s="11" t="str"/>
-      <x:c r="J8" s="11" t="str">
+      <x:c r="I8" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K8" s="11"/>
-      <x:c r="L8" s="11"/>
+      <x:c r="J8" s="11" t="str"/>
+      <x:c r="K8" s="11" t="str"/>
+      <x:c r="L8" s="11" t="str"/>
       <x:c r="M8" s="11" t="str"/>
       <x:c r="N8" s="11" t="str"/>
       <x:c r="P8" s="11" t="inlineStr">
@@ -4923,12 +4923,12 @@
           <x:t xml:space="preserve">STT 원문이 요약문만으로 대체되지 않음을 보여줌</x:t>
         </x:is>
       </x:c>
-      <x:c r="I9" s="11" t="str"/>
-      <x:c r="J9" s="11" t="str">
+      <x:c r="I9" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K9" s="11"/>
-      <x:c r="L9" s="11"/>
+      <x:c r="J9" s="11" t="str"/>
+      <x:c r="K9" s="11" t="str"/>
+      <x:c r="L9" s="11" t="str"/>
       <x:c r="M9" s="11" t="str"/>
       <x:c r="N9" s="11" t="str"/>
       <x:c r="P9" s="11" t="inlineStr">
@@ -4981,12 +4981,12 @@
           <x:t xml:space="preserve">학습 행동 지침</x:t>
         </x:is>
       </x:c>
-      <x:c r="I10" s="11" t="str"/>
-      <x:c r="J10" s="11" t="str">
+      <x:c r="I10" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K10" s="11"/>
-      <x:c r="L10" s="11"/>
+      <x:c r="J10" s="11" t="str"/>
+      <x:c r="K10" s="11" t="str"/>
+      <x:c r="L10" s="11" t="str"/>
       <x:c r="M10" s="11" t="str"/>
       <x:c r="N10" s="11" t="str"/>
     </x:row>
@@ -5029,12 +5029,12 @@
           <x:t xml:space="preserve">리뷰 행동에 직접 적용</x:t>
         </x:is>
       </x:c>
-      <x:c r="I11" s="11" t="str"/>
-      <x:c r="J11" s="11" t="str">
+      <x:c r="I11" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K11" s="11"/>
-      <x:c r="L11" s="11"/>
+      <x:c r="J11" s="11" t="str"/>
+      <x:c r="K11" s="11" t="str"/>
+      <x:c r="L11" s="11" t="str"/>
       <x:c r="M11" s="11" t="str"/>
       <x:c r="N11" s="11" t="str"/>
     </x:row>
@@ -5077,16 +5077,16 @@
           <x:t xml:space="preserve">실무 맥락 연결</x:t>
         </x:is>
       </x:c>
-      <x:c r="I12" s="11" t="str"/>
+      <x:c r="I12" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J12" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K12" s="11" t="str">
-        <x:v>실무적용</x:v>
-      </x:c>
-      <x:c r="L12" s="11" t="n">
+        <x:v>PRACTICAL</x:v>
+      </x:c>
+      <x:c r="K12" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L12" s="11" t="str"/>
       <x:c r="M12" s="11" t="str"/>
       <x:c r="N12" s="11" t="str"/>
     </x:row>
@@ -5129,12 +5129,12 @@
           <x:t xml:space="preserve">질문·검증 행동 유도</x:t>
         </x:is>
       </x:c>
-      <x:c r="I13" s="11" t="str"/>
-      <x:c r="J13" s="11" t="str">
+      <x:c r="I13" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K13" s="11"/>
-      <x:c r="L13" s="11"/>
+      <x:c r="J13" s="11" t="str"/>
+      <x:c r="K13" s="11" t="str"/>
+      <x:c r="L13" s="11" t="str"/>
       <x:c r="M13" s="11" t="str"/>
       <x:c r="N13" s="11" t="str"/>
     </x:row>
@@ -5177,12 +5177,12 @@
           <x:t xml:space="preserve">추가 학습 경로</x:t>
         </x:is>
       </x:c>
-      <x:c r="I14" s="11" t="str"/>
-      <x:c r="J14" s="11" t="str">
+      <x:c r="I14" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K14" s="11"/>
-      <x:c r="L14" s="11"/>
+      <x:c r="J14" s="11" t="str"/>
+      <x:c r="K14" s="11" t="str"/>
+      <x:c r="L14" s="11" t="str"/>
       <x:c r="M14" s="11" t="str"/>
       <x:c r="N14" s="11" t="str"/>
     </x:row>
@@ -5225,12 +5225,12 @@
           <x:t xml:space="preserve">교육에서의 핵심 인사이트</x:t>
         </x:is>
       </x:c>
-      <x:c r="I15" s="11" t="str"/>
-      <x:c r="J15" s="11" t="str">
+      <x:c r="I15" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K15" s="11"/>
-      <x:c r="L15" s="11"/>
+      <x:c r="J15" s="11" t="str"/>
+      <x:c r="K15" s="11" t="str"/>
+      <x:c r="L15" s="11" t="str"/>
       <x:c r="M15" s="11" t="str"/>
       <x:c r="N15" s="11" t="str"/>
     </x:row>
@@ -5273,16 +5273,16 @@
           <x:t xml:space="preserve">PM 사고방식의 핵심 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I16" s="11" t="str"/>
+      <x:c r="I16" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J16" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K16" s="11" t="str">
-        <x:v>주의·금지</x:v>
-      </x:c>
-      <x:c r="L16" s="11" t="n">
+        <x:v>AVOID</x:v>
+      </x:c>
+      <x:c r="K16" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L16" s="11" t="str"/>
       <x:c r="M16" s="11" t="str"/>
       <x:c r="N16" s="11" t="str"/>
     </x:row>
@@ -5325,12 +5325,12 @@
           <x:t xml:space="preserve">학습 행동 지침</x:t>
         </x:is>
       </x:c>
-      <x:c r="I17" s="11" t="str"/>
-      <x:c r="J17" s="11" t="str">
+      <x:c r="I17" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K17" s="11"/>
-      <x:c r="L17" s="11"/>
+      <x:c r="J17" s="11" t="str"/>
+      <x:c r="K17" s="11" t="str"/>
+      <x:c r="L17" s="11" t="str"/>
       <x:c r="M17" s="11" t="str"/>
       <x:c r="N17" s="11" t="str"/>
     </x:row>
@@ -5373,16 +5373,16 @@
           <x:t xml:space="preserve">AI 산출물 검수 포인트</x:t>
         </x:is>
       </x:c>
-      <x:c r="I18" s="11" t="str"/>
+      <x:c r="I18" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J18" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K18" s="11" t="str">
-        <x:v>주의·금지</x:v>
-      </x:c>
-      <x:c r="L18" s="11" t="n">
+        <x:v>AVOID</x:v>
+      </x:c>
+      <x:c r="K18" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L18" s="11" t="str"/>
       <x:c r="M18" s="11" t="str"/>
       <x:c r="N18" s="11" t="str"/>
     </x:row>
@@ -5425,12 +5425,12 @@
           <x:t xml:space="preserve">프로세스 핵심</x:t>
         </x:is>
       </x:c>
-      <x:c r="I19" s="11" t="str"/>
-      <x:c r="J19" s="11" t="str">
+      <x:c r="I19" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K19" s="11"/>
-      <x:c r="L19" s="11"/>
+      <x:c r="J19" s="11" t="str"/>
+      <x:c r="K19" s="11" t="str"/>
+      <x:c r="L19" s="11" t="str"/>
       <x:c r="M19" s="11" t="str"/>
       <x:c r="N19" s="11" t="str"/>
     </x:row>
@@ -5473,16 +5473,16 @@
           <x:t xml:space="preserve">PM 실무 판단 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I20" s="11" t="str"/>
+      <x:c r="I20" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J20" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K20" s="11" t="str">
-        <x:v>실무적용</x:v>
-      </x:c>
-      <x:c r="L20" s="11" t="n">
+        <x:v>PRACTICAL</x:v>
+      </x:c>
+      <x:c r="K20" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L20" s="11" t="str"/>
       <x:c r="M20" s="11" t="str"/>
       <x:c r="N20" s="11" t="str"/>
     </x:row>
@@ -5525,16 +5525,16 @@
           <x:t xml:space="preserve">작업 방식 주의</x:t>
         </x:is>
       </x:c>
-      <x:c r="I21" s="11" t="str"/>
+      <x:c r="I21" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J21" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K21" s="11" t="str">
-        <x:v>실무적용</x:v>
-      </x:c>
-      <x:c r="L21" s="11" t="n">
+        <x:v>PRACTICAL</x:v>
+      </x:c>
+      <x:c r="K21" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L21" s="11" t="str"/>
       <x:c r="M21" s="11" t="str"/>
       <x:c r="N21" s="11" t="str"/>
     </x:row>
@@ -5577,12 +5577,12 @@
           <x:t xml:space="preserve">최종 산출물 품질 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I22" s="11" t="str"/>
-      <x:c r="J22" s="11" t="str">
+      <x:c r="I22" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K22" s="11"/>
-      <x:c r="L22" s="11"/>
+      <x:c r="J22" s="11" t="str"/>
+      <x:c r="K22" s="11" t="str"/>
+      <x:c r="L22" s="11" t="str"/>
       <x:c r="M22" s="11" t="str"/>
       <x:c r="N22" s="11" t="str"/>
     </x:row>
@@ -5625,16 +5625,16 @@
           <x:t xml:space="preserve">MVP 구현 전략</x:t>
         </x:is>
       </x:c>
-      <x:c r="I23" s="11" t="str"/>
+      <x:c r="I23" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J23" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K23" s="11" t="str">
-        <x:v>실무적용</x:v>
-      </x:c>
-      <x:c r="L23" s="11" t="n">
+        <x:v>PRACTICAL</x:v>
+      </x:c>
+      <x:c r="K23" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L23" s="11" t="str"/>
       <x:c r="M23" s="11" t="str"/>
       <x:c r="N23" s="11" t="str"/>
     </x:row>
@@ -5677,16 +5677,16 @@
           <x:t xml:space="preserve">에이전트 설계 인사이트</x:t>
         </x:is>
       </x:c>
-      <x:c r="I24" s="11" t="str"/>
+      <x:c r="I24" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J24" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K24" s="11" t="str">
-        <x:v>핵심원칙</x:v>
-      </x:c>
-      <x:c r="L24" s="11" t="n">
+        <x:v>CORE</x:v>
+      </x:c>
+      <x:c r="K24" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L24" s="11" t="str"/>
       <x:c r="M24" s="11" t="str"/>
       <x:c r="N24" s="11" t="str"/>
     </x:row>
@@ -5729,12 +5729,12 @@
           <x:t xml:space="preserve">현실적인 일정 산정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I25" s="11" t="str"/>
-      <x:c r="J25" s="11" t="str">
+      <x:c r="I25" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K25" s="11"/>
-      <x:c r="L25" s="11"/>
+      <x:c r="J25" s="11" t="str"/>
+      <x:c r="K25" s="11" t="str"/>
+      <x:c r="L25" s="11" t="str"/>
       <x:c r="M25" s="11" t="str"/>
       <x:c r="N25" s="11" t="str"/>
     </x:row>
@@ -5777,12 +5777,12 @@
           <x:t xml:space="preserve">AI 산출물 비판적 검토</x:t>
         </x:is>
       </x:c>
-      <x:c r="I26" s="11" t="str"/>
-      <x:c r="J26" s="11" t="str">
+      <x:c r="I26" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K26" s="11"/>
-      <x:c r="L26" s="11"/>
+      <x:c r="J26" s="11" t="str"/>
+      <x:c r="K26" s="11" t="str"/>
+      <x:c r="L26" s="11" t="str"/>
       <x:c r="M26" s="11" t="str"/>
       <x:c r="N26" s="11" t="str"/>
     </x:row>
@@ -5825,12 +5825,12 @@
           <x:t xml:space="preserve">명시적 가치 부여</x:t>
         </x:is>
       </x:c>
-      <x:c r="I27" s="11" t="str"/>
-      <x:c r="J27" s="11" t="str">
+      <x:c r="I27" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K27" s="11"/>
-      <x:c r="L27" s="11"/>
+      <x:c r="J27" s="11" t="str"/>
+      <x:c r="K27" s="11" t="str"/>
+      <x:c r="L27" s="11" t="str"/>
       <x:c r="M27" s="11" t="str"/>
       <x:c r="N27" s="11" t="str"/>
     </x:row>
@@ -5873,16 +5873,16 @@
           <x:t xml:space="preserve">일정 최적화</x:t>
         </x:is>
       </x:c>
-      <x:c r="I28" s="11" t="str"/>
+      <x:c r="I28" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J28" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K28" s="11" t="str">
-        <x:v>주의·금지</x:v>
-      </x:c>
-      <x:c r="L28" s="11" t="n">
+        <x:v>AVOID</x:v>
+      </x:c>
+      <x:c r="K28" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L28" s="11" t="str"/>
       <x:c r="M28" s="11" t="str"/>
       <x:c r="N28" s="11" t="str"/>
     </x:row>
@@ -5925,12 +5925,12 @@
           <x:t xml:space="preserve">PM 핵심 질문</x:t>
         </x:is>
       </x:c>
-      <x:c r="I29" s="11" t="str"/>
-      <x:c r="J29" s="11" t="str">
+      <x:c r="I29" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K29" s="11"/>
-      <x:c r="L29" s="11"/>
+      <x:c r="J29" s="11" t="str"/>
+      <x:c r="K29" s="11" t="str"/>
+      <x:c r="L29" s="11" t="str"/>
       <x:c r="M29" s="11" t="str"/>
       <x:c r="N29" s="11" t="str"/>
     </x:row>
@@ -5973,16 +5973,16 @@
           <x:t xml:space="preserve">근거 기반 커뮤니케이션</x:t>
         </x:is>
       </x:c>
-      <x:c r="I30" s="11" t="str"/>
+      <x:c r="I30" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J30" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K30" s="11" t="str">
-        <x:v>실무적용</x:v>
-      </x:c>
-      <x:c r="L30" s="11" t="n">
+        <x:v>PRACTICAL</x:v>
+      </x:c>
+      <x:c r="K30" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L30" s="11" t="str"/>
       <x:c r="M30" s="11" t="str"/>
       <x:c r="N30" s="11" t="str"/>
     </x:row>
@@ -6025,12 +6025,12 @@
           <x:t xml:space="preserve">프롬프트/프로젝트 컨텍스트 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I31" s="11" t="str"/>
-      <x:c r="J31" s="11" t="str">
+      <x:c r="I31" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K31" s="11"/>
-      <x:c r="L31" s="11"/>
+      <x:c r="J31" s="11" t="str"/>
+      <x:c r="K31" s="11" t="str"/>
+      <x:c r="L31" s="11" t="str"/>
       <x:c r="M31" s="11" t="str"/>
       <x:c r="N31" s="11" t="str"/>
     </x:row>
@@ -6073,12 +6073,12 @@
           <x:t xml:space="preserve">도구 선택 판단</x:t>
         </x:is>
       </x:c>
-      <x:c r="I32" s="11" t="str"/>
-      <x:c r="J32" s="11" t="str">
+      <x:c r="I32" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K32" s="11"/>
-      <x:c r="L32" s="11"/>
+      <x:c r="J32" s="11" t="str"/>
+      <x:c r="K32" s="11" t="str"/>
+      <x:c r="L32" s="11" t="str"/>
       <x:c r="M32" s="11" t="str"/>
       <x:c r="N32" s="11" t="str"/>
     </x:row>
@@ -6121,12 +6121,12 @@
           <x:t xml:space="preserve">PM-엔지니어링 결합 역량</x:t>
         </x:is>
       </x:c>
-      <x:c r="I33" s="11" t="str"/>
-      <x:c r="J33" s="11" t="str">
+      <x:c r="I33" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K33" s="11"/>
-      <x:c r="L33" s="11"/>
+      <x:c r="J33" s="11" t="str"/>
+      <x:c r="K33" s="11" t="str"/>
+      <x:c r="L33" s="11" t="str"/>
       <x:c r="M33" s="11" t="str"/>
       <x:c r="N33" s="11" t="str"/>
     </x:row>
@@ -6169,16 +6169,16 @@
           <x:t xml:space="preserve">메타 역량</x:t>
         </x:is>
       </x:c>
-      <x:c r="I34" s="11" t="str"/>
+      <x:c r="I34" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J34" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K34" s="11" t="str">
-        <x:v>핵심원칙</x:v>
-      </x:c>
-      <x:c r="L34" s="11" t="n">
+        <x:v>CORE</x:v>
+      </x:c>
+      <x:c r="K34" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L34" s="11" t="str"/>
       <x:c r="M34" s="11" t="str"/>
       <x:c r="N34" s="11" t="str"/>
     </x:row>
@@ -6221,16 +6221,16 @@
           <x:t xml:space="preserve">AI-native 작업 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I35" s="11" t="str"/>
+      <x:c r="I35" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J35" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K35" s="11" t="str">
-        <x:v>핵심원칙</x:v>
-      </x:c>
-      <x:c r="L35" s="11" t="n">
+        <x:v>CORE</x:v>
+      </x:c>
+      <x:c r="K35" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L35" s="11" t="str"/>
       <x:c r="M35" s="11" t="str"/>
       <x:c r="N35" s="11" t="str"/>
     </x:row>
@@ -6273,12 +6273,12 @@
           <x:t xml:space="preserve">AI-native 작업 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I36" s="11" t="str"/>
-      <x:c r="J36" s="11" t="str">
+      <x:c r="I36" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K36" s="11"/>
-      <x:c r="L36" s="11"/>
+      <x:c r="J36" s="11" t="str"/>
+      <x:c r="K36" s="11" t="str"/>
+      <x:c r="L36" s="11" t="str"/>
       <x:c r="M36" s="11" t="str"/>
       <x:c r="N36" s="11" t="str"/>
     </x:row>
@@ -6321,12 +6321,12 @@
           <x:t xml:space="preserve">실험 설계 전제</x:t>
         </x:is>
       </x:c>
-      <x:c r="I37" s="11" t="str"/>
-      <x:c r="J37" s="11" t="str">
+      <x:c r="I37" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K37" s="11"/>
-      <x:c r="L37" s="11"/>
+      <x:c r="J37" s="11" t="str"/>
+      <x:c r="K37" s="11" t="str"/>
+      <x:c r="L37" s="11" t="str"/>
       <x:c r="M37" s="11" t="str"/>
       <x:c r="N37" s="11" t="str"/>
     </x:row>
@@ -6369,12 +6369,12 @@
           <x:t xml:space="preserve">실행 전제</x:t>
         </x:is>
       </x:c>
-      <x:c r="I38" s="11" t="str"/>
-      <x:c r="J38" s="11" t="str">
+      <x:c r="I38" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K38" s="11"/>
-      <x:c r="L38" s="11"/>
+      <x:c r="J38" s="11" t="str"/>
+      <x:c r="K38" s="11" t="str"/>
+      <x:c r="L38" s="11" t="str"/>
       <x:c r="M38" s="11" t="str"/>
       <x:c r="N38" s="11" t="str"/>
     </x:row>
@@ -6417,16 +6417,16 @@
           <x:t xml:space="preserve">검증 방법</x:t>
         </x:is>
       </x:c>
-      <x:c r="I39" s="11" t="str"/>
+      <x:c r="I39" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J39" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K39" s="11" t="str">
-        <x:v>핵심원칙</x:v>
-      </x:c>
-      <x:c r="L39" s="11" t="n">
+        <x:v>CORE</x:v>
+      </x:c>
+      <x:c r="K39" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L39" s="11" t="str"/>
       <x:c r="M39" s="11" t="str"/>
       <x:c r="N39" s="11" t="str"/>
     </x:row>
@@ -6469,16 +6469,16 @@
           <x:t xml:space="preserve">에이전트 인터뷰 기록</x:t>
         </x:is>
       </x:c>
-      <x:c r="I40" s="11" t="str"/>
+      <x:c r="I40" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J40" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K40" s="11" t="str">
-        <x:v>핵심원칙</x:v>
-      </x:c>
-      <x:c r="L40" s="11" t="n">
+        <x:v>CORE</x:v>
+      </x:c>
+      <x:c r="K40" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L40" s="11" t="str"/>
       <x:c r="M40" s="11" t="str"/>
       <x:c r="N40" s="11" t="str"/>
     </x:row>
@@ -6521,12 +6521,12 @@
           <x:t xml:space="preserve">기획→구현 연결</x:t>
         </x:is>
       </x:c>
-      <x:c r="I41" s="11" t="str"/>
-      <x:c r="J41" s="11" t="str">
+      <x:c r="I41" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K41" s="11"/>
-      <x:c r="L41" s="11"/>
+      <x:c r="J41" s="11" t="str"/>
+      <x:c r="K41" s="11" t="str"/>
+      <x:c r="L41" s="11" t="str"/>
       <x:c r="M41" s="11" t="str"/>
       <x:c r="N41" s="11" t="str"/>
     </x:row>
@@ -6569,12 +6569,12 @@
           <x:t xml:space="preserve">에이전트 제어 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I42" s="11" t="str"/>
-      <x:c r="J42" s="11" t="str">
+      <x:c r="I42" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K42" s="11"/>
-      <x:c r="L42" s="11"/>
+      <x:c r="J42" s="11" t="str"/>
+      <x:c r="K42" s="11" t="str"/>
+      <x:c r="L42" s="11" t="str"/>
       <x:c r="M42" s="11" t="str"/>
       <x:c r="N42" s="11" t="str"/>
     </x:row>
@@ -6617,12 +6617,12 @@
           <x:t xml:space="preserve">에이전트 투명성</x:t>
         </x:is>
       </x:c>
-      <x:c r="I43" s="11" t="str"/>
-      <x:c r="J43" s="11" t="str">
+      <x:c r="I43" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K43" s="11"/>
-      <x:c r="L43" s="11"/>
+      <x:c r="J43" s="11" t="str"/>
+      <x:c r="K43" s="11" t="str"/>
+      <x:c r="L43" s="11" t="str"/>
       <x:c r="M43" s="11" t="str"/>
       <x:c r="N43" s="11" t="str"/>
     </x:row>
@@ -6665,12 +6665,12 @@
           <x:t xml:space="preserve">오너십/추적성</x:t>
         </x:is>
       </x:c>
-      <x:c r="I44" s="11" t="str"/>
-      <x:c r="J44" s="11" t="str">
+      <x:c r="I44" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K44" s="11"/>
-      <x:c r="L44" s="11"/>
+      <x:c r="J44" s="11" t="str"/>
+      <x:c r="K44" s="11" t="str"/>
+      <x:c r="L44" s="11" t="str"/>
       <x:c r="M44" s="11" t="str"/>
       <x:c r="N44" s="11" t="str"/>
     </x:row>
@@ -6713,12 +6713,12 @@
           <x:t xml:space="preserve">프로토타입 품질 기준</x:t>
         </x:is>
       </x:c>
-      <x:c r="I45" s="11" t="str"/>
-      <x:c r="J45" s="11" t="str">
+      <x:c r="I45" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K45" s="11"/>
-      <x:c r="L45" s="11"/>
+      <x:c r="J45" s="11" t="str"/>
+      <x:c r="K45" s="11" t="str"/>
+      <x:c r="L45" s="11" t="str"/>
       <x:c r="M45" s="11" t="str"/>
       <x:c r="N45" s="11" t="str"/>
     </x:row>
@@ -6761,16 +6761,16 @@
           <x:t xml:space="preserve">완성 조건</x:t>
         </x:is>
       </x:c>
-      <x:c r="I46" s="11" t="str"/>
+      <x:c r="I46" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J46" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K46" s="11" t="str">
-        <x:v>강조</x:v>
-      </x:c>
-      <x:c r="L46" s="11" t="n">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K46" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L46" s="11" t="str"/>
       <x:c r="M46" s="11" t="str"/>
       <x:c r="N46" s="11" t="str"/>
     </x:row>
@@ -6813,12 +6813,12 @@
           <x:t xml:space="preserve">에이전트 거버넌스</x:t>
         </x:is>
       </x:c>
-      <x:c r="I47" s="11" t="str"/>
-      <x:c r="J47" s="11" t="str">
+      <x:c r="I47" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K47" s="11"/>
-      <x:c r="L47" s="11"/>
+      <x:c r="J47" s="11" t="str"/>
+      <x:c r="K47" s="11" t="str"/>
+      <x:c r="L47" s="11" t="str"/>
       <x:c r="M47" s="11" t="str"/>
       <x:c r="N47" s="11" t="str"/>
     </x:row>
@@ -6861,12 +6861,12 @@
           <x:t xml:space="preserve">AI-native 운영 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I48" s="11" t="str"/>
-      <x:c r="J48" s="11" t="str">
+      <x:c r="I48" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K48" s="11"/>
-      <x:c r="L48" s="11"/>
+      <x:c r="J48" s="11" t="str"/>
+      <x:c r="K48" s="11" t="str"/>
+      <x:c r="L48" s="11" t="str"/>
       <x:c r="M48" s="11" t="str"/>
       <x:c r="N48" s="11" t="str"/>
     </x:row>
@@ -6909,12 +6909,12 @@
           <x:t xml:space="preserve">자율성 정량화</x:t>
         </x:is>
       </x:c>
-      <x:c r="I49" s="11" t="str"/>
-      <x:c r="J49" s="11" t="str">
+      <x:c r="I49" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K49" s="11"/>
-      <x:c r="L49" s="11"/>
+      <x:c r="J49" s="11" t="str"/>
+      <x:c r="K49" s="11" t="str"/>
+      <x:c r="L49" s="11" t="str"/>
       <x:c r="M49" s="11" t="str"/>
       <x:c r="N49" s="11" t="str"/>
     </x:row>
@@ -6957,16 +6957,16 @@
           <x:t xml:space="preserve">사후 제어 규칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I50" s="11" t="str"/>
+      <x:c r="I50" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J50" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K50" s="11" t="str">
-        <x:v>주의·금지</x:v>
-      </x:c>
-      <x:c r="L50" s="11" t="n">
+        <x:v>AVOID</x:v>
+      </x:c>
+      <x:c r="K50" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="L50" s="11" t="str"/>
       <x:c r="M50" s="11" t="str"/>
       <x:c r="N50" s="11" t="str"/>
     </x:row>
@@ -7009,12 +7009,12 @@
           <x:t xml:space="preserve">위험도 기반 자율성</x:t>
         </x:is>
       </x:c>
-      <x:c r="I51" s="11" t="str"/>
-      <x:c r="J51" s="11" t="str">
+      <x:c r="I51" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K51" s="11"/>
-      <x:c r="L51" s="11"/>
+      <x:c r="J51" s="11" t="str"/>
+      <x:c r="K51" s="11" t="str"/>
+      <x:c r="L51" s="11" t="str"/>
       <x:c r="M51" s="11" t="str"/>
       <x:c r="N51" s="11" t="str"/>
     </x:row>
@@ -7057,12 +7057,12 @@
           <x:t xml:space="preserve">생산성/통제 균형</x:t>
         </x:is>
       </x:c>
-      <x:c r="I52" s="11" t="str"/>
-      <x:c r="J52" s="11" t="str">
+      <x:c r="I52" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K52" s="11"/>
-      <x:c r="L52" s="11"/>
+      <x:c r="J52" s="11" t="str"/>
+      <x:c r="K52" s="11" t="str"/>
+      <x:c r="L52" s="11" t="str"/>
       <x:c r="M52" s="11" t="str"/>
       <x:c r="N52" s="11" t="str"/>
     </x:row>
@@ -7105,12 +7105,12 @@
           <x:t xml:space="preserve">정량적 관리</x:t>
         </x:is>
       </x:c>
-      <x:c r="I53" s="11" t="str"/>
-      <x:c r="J53" s="11" t="str">
+      <x:c r="I53" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K53" s="11"/>
-      <x:c r="L53" s="11"/>
+      <x:c r="J53" s="11" t="str"/>
+      <x:c r="K53" s="11" t="str"/>
+      <x:c r="L53" s="11" t="str"/>
       <x:c r="M53" s="11" t="str"/>
       <x:c r="N53" s="11" t="str"/>
     </x:row>
@@ -7153,16 +7153,16 @@
           <x:t xml:space="preserve">에이전트 작업 설계</x:t>
         </x:is>
       </x:c>
-      <x:c r="I54" s="11" t="str"/>
+      <x:c r="I54" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J54" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K54" s="11" t="str">
-        <x:v>강조</x:v>
-      </x:c>
-      <x:c r="L54" s="11" t="n">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K54" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L54" s="11" t="str"/>
       <x:c r="M54" s="11" t="str"/>
       <x:c r="N54" s="11" t="str"/>
     </x:row>
@@ -7205,12 +7205,12 @@
           <x:t xml:space="preserve">작업량 추정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I55" s="11" t="str"/>
-      <x:c r="J55" s="11" t="str">
+      <x:c r="I55" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K55" s="11"/>
-      <x:c r="L55" s="11"/>
+      <x:c r="J55" s="11" t="str"/>
+      <x:c r="K55" s="11" t="str"/>
+      <x:c r="L55" s="11" t="str"/>
       <x:c r="M55" s="11" t="str"/>
       <x:c r="N55" s="11" t="str"/>
     </x:row>
@@ -7253,12 +7253,12 @@
           <x:t xml:space="preserve">에이전트 예산 관리</x:t>
         </x:is>
       </x:c>
-      <x:c r="I56" s="11" t="str"/>
-      <x:c r="J56" s="11" t="str">
+      <x:c r="I56" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K56" s="11"/>
-      <x:c r="L56" s="11"/>
+      <x:c r="J56" s="11" t="str"/>
+      <x:c r="K56" s="11" t="str"/>
+      <x:c r="L56" s="11" t="str"/>
       <x:c r="M56" s="11" t="str"/>
       <x:c r="N56" s="11" t="str"/>
     </x:row>
@@ -7301,12 +7301,12 @@
           <x:t xml:space="preserve">에이전트 예산</x:t>
         </x:is>
       </x:c>
-      <x:c r="I57" s="11" t="str"/>
-      <x:c r="J57" s="11" t="str">
+      <x:c r="I57" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K57" s="11"/>
-      <x:c r="L57" s="11"/>
+      <x:c r="J57" s="11" t="str"/>
+      <x:c r="K57" s="11" t="str"/>
+      <x:c r="L57" s="11" t="str"/>
       <x:c r="M57" s="11" t="str"/>
       <x:c r="N57" s="11" t="str"/>
     </x:row>
@@ -7349,12 +7349,12 @@
           <x:t xml:space="preserve">프로토타이핑 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I58" s="11" t="str"/>
-      <x:c r="J58" s="11" t="str">
+      <x:c r="I58" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K58" s="11"/>
-      <x:c r="L58" s="11"/>
+      <x:c r="J58" s="11" t="str"/>
+      <x:c r="K58" s="11" t="str"/>
+      <x:c r="L58" s="11" t="str"/>
       <x:c r="M58" s="11" t="str"/>
       <x:c r="N58" s="11" t="str"/>
     </x:row>
@@ -7397,16 +7397,16 @@
           <x:t xml:space="preserve">반복 개선 태도</x:t>
         </x:is>
       </x:c>
-      <x:c r="I59" s="11" t="str"/>
+      <x:c r="I59" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J59" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K59" s="11" t="str">
-        <x:v>강조</x:v>
-      </x:c>
-      <x:c r="L59" s="11" t="n">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K59" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L59" s="11" t="str"/>
       <x:c r="M59" s="11" t="str"/>
       <x:c r="N59" s="11" t="str"/>
     </x:row>
@@ -7449,16 +7449,16 @@
           <x:t xml:space="preserve">서비스→GTM 연결</x:t>
         </x:is>
       </x:c>
-      <x:c r="I60" s="11" t="str"/>
+      <x:c r="I60" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
       <x:c r="J60" s="11" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="K60" s="11" t="str">
-        <x:v>강조</x:v>
-      </x:c>
-      <x:c r="L60" s="11" t="n">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K60" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="L60" s="11" t="str"/>
       <x:c r="M60" s="11" t="str"/>
       <x:c r="N60" s="11" t="str"/>
     </x:row>
@@ -7501,12 +7501,12 @@
           <x:t xml:space="preserve">전환 설계</x:t>
         </x:is>
       </x:c>
-      <x:c r="I61" s="11" t="str"/>
-      <x:c r="J61" s="11" t="str">
+      <x:c r="I61" s="11" t="str">
         <x:v>N</x:v>
       </x:c>
-      <x:c r="K61" s="11"/>
-      <x:c r="L61" s="11"/>
+      <x:c r="J61" s="11" t="str"/>
+      <x:c r="K61" s="11" t="str"/>
+      <x:c r="L61" s="11" t="str"/>
       <x:c r="M61" s="11" t="str"/>
       <x:c r="N61" s="11" t="str"/>
     </x:row>
@@ -7549,7 +7549,9 @@
           <x:t xml:space="preserve">서비스별 증거 설계</x:t>
         </x:is>
       </x:c>
-      <x:c r="I62" s="11" t="str"/>
+      <x:c r="I62" s="11" t="str">
+        <x:v>N</x:v>
+      </x:c>
       <x:c r="J62" s="11" t="str"/>
       <x:c r="K62" s="11" t="str"/>
       <x:c r="L62" s="11" t="str"/>
@@ -7595,7 +7597,9 @@
           <x:t xml:space="preserve">전환의 근거</x:t>
         </x:is>
       </x:c>
-      <x:c r="I63" s="11" t="str"/>
+      <x:c r="I63" s="11" t="str">
+        <x:v>N</x:v>
+      </x:c>
       <x:c r="J63" s="11" t="str"/>
       <x:c r="K63" s="11" t="str"/>
       <x:c r="L63" s="11" t="str"/>
@@ -7641,9 +7645,15 @@
           <x:t xml:space="preserve">퍼널 핵심 원칙</x:t>
         </x:is>
       </x:c>
-      <x:c r="I64" s="11" t="str"/>
-      <x:c r="J64" s="11" t="str"/>
-      <x:c r="K64" s="11" t="str"/>
+      <x:c r="I64" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J64" s="11" t="str">
+        <x:v>CORE</x:v>
+      </x:c>
+      <x:c r="K64" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="L64" s="11" t="str"/>
       <x:c r="M64" s="11" t="str"/>
       <x:c r="N64" s="11" t="str"/>
@@ -7687,9 +7697,15 @@
           <x:t xml:space="preserve">리스크 커뮤니케이션</x:t>
         </x:is>
       </x:c>
-      <x:c r="I65" s="11" t="str"/>
-      <x:c r="J65" s="11" t="str"/>
-      <x:c r="K65" s="11" t="str"/>
+      <x:c r="I65" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J65" s="11" t="str">
+        <x:v>AVOID</x:v>
+      </x:c>
+      <x:c r="K65" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="L65" s="11" t="str"/>
       <x:c r="M65" s="11" t="str"/>
       <x:c r="N65" s="11" t="str"/>
@@ -7733,7 +7749,9 @@
           <x:t xml:space="preserve">데이터 검증</x:t>
         </x:is>
       </x:c>
-      <x:c r="I66" s="11" t="str"/>
+      <x:c r="I66" s="11" t="str">
+        <x:v>N</x:v>
+      </x:c>
       <x:c r="J66" s="11" t="str"/>
       <x:c r="K66" s="11" t="str"/>
       <x:c r="L66" s="11" t="str"/>
@@ -7779,9 +7797,15 @@
           <x:t xml:space="preserve">정확한 수정 지시</x:t>
         </x:is>
       </x:c>
-      <x:c r="I67" s="11" t="str"/>
-      <x:c r="J67" s="11" t="str"/>
-      <x:c r="K67" s="11" t="str"/>
+      <x:c r="I67" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J67" s="11" t="str">
+        <x:v>EMPHASIS</x:v>
+      </x:c>
+      <x:c r="K67" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="L67" s="11" t="str"/>
       <x:c r="M67" s="11" t="str"/>
       <x:c r="N67" s="11" t="str"/>
@@ -7825,9 +7849,15 @@
           <x:t xml:space="preserve">AI 구현 품질</x:t>
         </x:is>
       </x:c>
-      <x:c r="I68" s="11" t="str"/>
-      <x:c r="J68" s="11" t="str"/>
-      <x:c r="K68" s="11" t="str"/>
+      <x:c r="I68" s="11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J68" s="11" t="str">
+        <x:v>AVOID</x:v>
+      </x:c>
+      <x:c r="K68" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="L68" s="11" t="str"/>
       <x:c r="M68" s="11" t="str"/>
       <x:c r="N68" s="11" t="str"/>
@@ -7871,7 +7901,9 @@
           <x:t xml:space="preserve">단계적 문제 해결</x:t>
         </x:is>
       </x:c>
-      <x:c r="I69" s="11" t="str"/>
+      <x:c r="I69" s="11" t="str">
+        <x:v>N</x:v>
+      </x:c>
       <x:c r="J69" s="11" t="str"/>
       <x:c r="K69" s="11" t="str"/>
       <x:c r="L69" s="11" t="str"/>

</xml_diff>

<commit_message>
chore(auto): save work in "\354\275\225\354\247\221 (1 file(s), 2026-09-11 13:57)
</commit_message>
<xml_diff>
--- a/콕집/KOKJIP_Signal_Dataset_v0.1_HumanReview.xlsx
+++ b/콕집/KOKJIP_Signal_Dataset_v0.1_HumanReview.xlsx
@@ -6,6 +6,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signal Dataset" sheetId="2" r:id="R2887ff91fd574893"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="3" r:id="Rf5401a04faf547c9"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Review" sheetId="4" r:id="R674c2ebd44c9471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Findings Review" sheetId="5" r:id="RnewFindings01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7913,4 +7914,2883 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="50" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="50" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="40" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">구분</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">날짜</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">타임스탬프(보정)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI 표기 타임스탬프</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">타임스탬프 보정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI Type</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI 강도</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI 요약</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">근거 발화</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">사람 판단 (Signal?)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">사람 판단 Type</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">사람 판단 강도</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O1" s="19" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">메모</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">03:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">03:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G2" s="11" t="str"/>
+      <x:c r="H2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I2" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">회고의 4단 구조: 왜/무엇을 했고/어떤 산출물을 얻었고/앞으로 어떻게</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">내가 왜? 무엇을 했고 어떤 산출물을 얻었고 앞으로 이걸 어떻게 하겠다라는 생각 정리</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L2" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M2" s="11" t="str"/>
+      <x:c r="N2" s="11" t="str"/>
+      <x:c r="O2" s="11" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">04:28</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">04:28</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G3" s="11" t="str"/>
+      <x:c r="H3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I3" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI에게 회고를 시킨 것은 인간이 회고한 것과 본질적으로 다름</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">인간이 회고해야 되는데 AI한테 회고한 것은 비슷한 게 아니죠? 아예 다른 거죠</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L3" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M3" s="11" t="str"/>
+      <x:c r="N3" s="11" t="str"/>
+      <x:c r="O3" s="11" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">05:37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">05:37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G4" s="11" t="str"/>
+      <x:c r="H4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I4" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">세부 항목부터가 아니라 전체 핵심 키워드로 아웃라인을 먼저 짤 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">전체 아웃라인을 먼저 짜 보면 또 어때요? 개념 지도가 부터 한번 쫙 펼쳐지고</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L4" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M4" s="11" t="str"/>
+      <x:c r="N4" s="11" t="str"/>
+      <x:c r="O4" s="11" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">08:18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">08:18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="11" t="str"/>
+      <x:c r="H5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I5" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRD 품질의 정의 — 루티드 문서, 기획 내용의 통합 원본</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRD는 루티드 문서여야 한다. 기획 내용의 통합 원본 역할을 해야 한다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M5" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N5" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O5" s="11" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">09:05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">09:05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="11" t="str"/>
+      <x:c r="H6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I6" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SRS는 표준 양식을 따르되 필요한 챕터만 간결히</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SRS는 표준 문서 양식을 따르되 필요한 챕터만 간결히 가져야 한다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M6" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">EMPHASIS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N6" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O6" s="11" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">09:44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">09:44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="11" t="str"/>
+      <x:c r="H7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I7" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">풀버전 표준문서를 쓰면 토큰·시간 비용이 폭증</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">토큰이 너무 많이 들고 항상 매번 뭐 칠 때마다 몇 십 분씩 걸려서</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M7" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N7" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O7" s="11" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">14:35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">15:03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">프로젝트 관리로 건너뛰고 싶어도 앞 단계에 시간을 쓴 이유가 있음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">그다음 단계로 프로젝트 관리로 갑자기 빨리 건너뛰고 싶겠지만 어제 충분한 시간을 쓴 이유가 있는 거죠</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L8" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M8" s="11" t="str"/>
+      <x:c r="N8" s="11" t="str"/>
+      <x:c r="O8" s="11" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N08</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">15:21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">15:21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="11" t="str"/>
+      <x:c r="H9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I9" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">교안에 외부 링크·레퍼런스를 다 넣으면 나중에 리뷰 시 방황하게 됨</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">다 들어가 있으면 좋다고 생각할 수도 있지만 여러분은 그러면 안 되거든요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M9" s="11" t="str"/>
+      <x:c r="N9" s="11" t="str"/>
+      <x:c r="O9" s="11" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">24:40</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">24:40</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="11" t="str"/>
+      <x:c r="H10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REVIEW</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I10" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">스크럼을 추가로 알아보고 리뷰를 풍성하게 할 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">추가로 좀 더 알아보고 여러분의 리뷰를 풍성하게 할 수가 있겠다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M10" s="11" t="str"/>
+      <x:c r="N10" s="11" t="str"/>
+      <x:c r="O10" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">회고 일괄 N 규칙 적용</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">37:26</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">37:26</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="11" t="str"/>
+      <x:c r="H11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I11" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">과잉 분할 시 통합이 아니라 상단 60개만 먼저 하는 방식으로 분할</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">그거는 그 작업을 통합하고 이렇게 하는 게 아니라 이번엔 위에 상단 먼저 하는 거 60개만</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRACTICAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N11" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O11" s="11" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">41:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">41:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="11" t="str"/>
+      <x:c r="H12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">한국어에 맞춘 다듬기를 시도하면 코딩 성능이 떨어짐 — 그러려니 하고 읽어야</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">그걸 한국말에 맞춰서 바람직한 국어로 다듬겠다라는 생각을 가지면 성능이 안 나와요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M12" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N12" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O12" s="11" t="str"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">46:22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">46:22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="11" t="str"/>
+      <x:c r="H13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">준비 안 된 외부 연동은 더미 데이터 생성이 아니라 API 모킹으로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">범위 데이터 생성해 줘. 워킹 해 줘. 그러지 마세요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRACTICAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N13" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">STT 오인식: 원문 음성은 '그렇게 하세요'(권장)인데 STT는 '그러지 마세요'(금지). AI가 이 오인식으로 AVOID 판정</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">48:25</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">47:37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">INSIGHT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I14" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">요구한 다이어그램이 안 나온 건 AI가 토큰을 절약한 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">얘가 이거를 안 뽑았다는 거는 사실 그 요구사항에 대해서 토큰 절약을 한 거야</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L14" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M14" s="11" t="str"/>
+      <x:c r="N14" s="11" t="str"/>
+      <x:c r="O14" s="11" t="str"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">50:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">50:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="11" t="str"/>
+      <x:c r="H15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I15" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">태스크는 한 시간 안에 끝나는 수준으로 썰려 있어야 함</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">한 시간 안에 끝나는 것들 수준으로 썰려 있어야 돼요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M15" s="11" t="str"/>
+      <x:c r="N15" s="11" t="str"/>
+      <x:c r="O15" s="11" t="str"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">53:46</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">53:46</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="11" t="str"/>
+      <x:c r="H16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I16" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DAG 노드 20개 초과 시 최대 30개 수준으로 축약 요청</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">최대 노드 30개의 수준으로 축약해서 표현해 줘라고 후속 프롬프팅</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M16" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRACTICAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N16" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O16" s="11" t="str"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">54:54</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">54:33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I17" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">노드 20개 정도가 사람이 읽을 수 있는 한계 — 넘으면 회의 자료로 못 씀</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">그 이상이 좀 넘어가기 시작하면 못 읽었고. 회의 자료로 쓸 수 없게</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N17" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O17" s="11" t="str"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N17</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:06:13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:06:13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" s="11" t="str"/>
+      <x:c r="H18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I18" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">예제 프롬프트의 파일명·링크는 반드시 본인 것으로 교체</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">여러분의 파일로 꼭 바꿔 줘야 된다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M18" s="11" t="str"/>
+      <x:c r="N18" s="11" t="str"/>
+      <x:c r="O18" s="11" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:23:27</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:23:27</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="11" t="str"/>
+      <x:c r="H19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I19" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CLI가 있는지를 먼저 확인하는 관점을 항상 가질 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CRI가 있는지를 먼저 확인하기 라는 관점을 여러분 항상 생각하면 좋겠어요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRACTICAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N19" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O19" s="11" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N19</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:25:15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:25:15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="11" t="str"/>
+      <x:c r="H20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">INSIGHT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I20" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI는 외부 통신 작업에서 보수적으로 최소만 함 — 최대한 하라고 명시해야</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">외부랑 통신해야 되는 부분이 있으면은 굉장히 좀 보수적으로 그 얘기한 만큼만</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M20" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRACTICAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N20" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O20" s="11" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:26:35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:26:35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" s="11" t="str"/>
+      <x:c r="H21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I21" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CLI 설치도 AI에게 시킬 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">네가 설치해라고 하세요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M21" s="11" t="str"/>
+      <x:c r="N21" s="11" t="str"/>
+      <x:c r="O21" s="11" t="str"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">27일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:08</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I22" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">수업 진도에 맞춰 다 뽑아놔야 한다는 방식으로 작업하면 안 됨</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">다 뽑아내고 그다음을 해야지라고 하는 느낌을 혹시 받는다면 그거 그런 식으로 뽑으면은 안 된다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L22" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M22" s="11" t="str"/>
+      <x:c r="N22" s="11" t="str"/>
+      <x:c r="O22" s="11" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">27일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">15:07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">15:30</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I23" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">그릴을 충분히 안 하면 미결정 영역을 AI가 알아서 처리하게 됨</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">내가 의사 결정하지 않은 부분에 대해서 얘가 알아서 작업하는 부분들이 많아질 것이다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N23" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O23" s="11" t="str"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N23</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">27일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">31:59</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">32:10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRACTICAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I24" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">골 프롬프트가 4000자를 넘으면 파일로 저장 후 참조</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">이거 파일로 저장한 다음에 볼 프롬프트에다가 이 파일에 있는 목표 달성할 때까지 해 줘</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M24" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PRACTICAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N24" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O24" s="11" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N24</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">27일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">50:39</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">51:02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I25" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">모든 프롬프트에 작업의 전·중·후를 그려보며 오너십을 확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업의 전 중후를 그려보면서 완벽하게 소유하고 있는가를 물어보면서 프롬프트를 한다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M25" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N25" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O25" s="11" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N25</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">27일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:03:45</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:03:20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">INSIGHT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I26" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI 슬롭은 다크테마 같은 시각요소가 아니라 언어의 문제</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">프로딩빙한 다크 테마가 다 문제가 아니라는 거예요. 언어적인 문제가 훨씬 더 크다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L26" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M26" s="11" t="str"/>
+      <x:c r="N26" s="11" t="str"/>
+      <x:c r="O26" s="11" t="str"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N26</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">27일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:20:04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:20:24</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I27" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">디스클레이머는 읽히는 폰트로 — 구석 작은 글씨는 바람직하지 않음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">디스클레이머 이거보다는 확실히 선명한 좀 밝은 폰트로 해야 돼요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M27" s="11" t="str"/>
+      <x:c r="N27" s="11" t="str"/>
+      <x:c r="O27" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI 요약 오류: '구석 작은 글씨는 바람직하지 않음'이라 요약했으나 원문(1:20:24)은 '구석에 작게 쓰는 것까지는 관계없다'로 반대 방향</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N27</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토구간 내 미탐</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">27일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">57:12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">57:02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I28" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">태스크 문서에 디자인 시스템이 이미 있어도 내 의도가 아니면 다시 세팅</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">포함되어 있어도 다시 놔야 됩니다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M28" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N28" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O28" s="11" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">21:30</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">21:30</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" s="11" t="str"/>
+      <x:c r="H29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I29" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI에게 프로젝트 구현 목표를 인식시켜 작업 규칙을 스스로 수립하게 함 = 메타인지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">그에 맞춰서 AI 작업 규칙을 네가 알아서 수립해라. 그 얘한테 메타 인지를 시키는 겁니다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M29" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N29" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O29" s="11" t="str"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">24:52</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">25:07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I30" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">프로젝트 핵심 목표를 오버뷰 규칙으로 잡으면 범위 이탈 작업이 줄어듦</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">이 프로젝트의 핵심 목표를 규칙으로 오버뷰로 잡아 놓는 방식을 따르면 이상한 게 안 들어가요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M30" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N30" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O30" s="11" t="str"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26:13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26:33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">RATIONALE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I31" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">하네스 샘플은 크게 만들어야 함 — 축약이 확장보다 토큰이 싸다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">있는 걸 축약하는 건 쉽거든. 토큰도 그게 더 절약되거든요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M31" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N31" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O31" s="11" t="str"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">37:24</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">37:24</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G32" s="11" t="str"/>
+      <x:c r="H32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I32" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">가져온 스킬은 인기 여부와 무관하게 반드시 열어보고 쓸 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">웬만해서는 내 프로젝트에 가져와서 쓰는 거는 다 열어 보고 써야 된다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N32" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O32" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">사용자 라벨 '주의' → AVOID 매핑</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">53:47</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">53:55</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I33" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">벤더가 제안하는 한 줄짜리 골 프롬프트로는 오너십이 생기지 않음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">절대 그거 해 그렇게 해서 오너십이 생기지 않아요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M33" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N33" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O33" s="11" t="str"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">54:33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">54:33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G34" s="11" t="str"/>
+      <x:c r="H34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I34" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">골을 바로 호출하지 말고 골 세팅 스킬을 먼저 호출</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">꼴이라고 호출하지 말고 제가 만드는 이 꼴 세팅 스킬을 호출해서</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L34" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M34" s="11" t="str"/>
+      <x:c r="N34" s="11" t="str"/>
+      <x:c r="O34" s="11" t="str"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:30:04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:29:57</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I35" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">랜딩 페이지의 본질은 다음 행동을 촉구하는 CTA 설계</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">어떤 행동을 하라고 촉구하는 디자인으로 돼 있어야 돼요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M35" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N35" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O35" s="11" t="str"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U08</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:40:38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:41:13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I36" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">이력서·포트폴리오·랜딩페이지 모두 각 섹션 제목을 정확히 뽑을 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">각 섹션의 제목을 정확하게 뽑으세요. 이력서든 포트폴리오든 랜딩 페이지든 다 마찬가지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M36" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N36" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O36" s="11" t="str"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:43:21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:43:21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G37" s="11" t="str"/>
+      <x:c r="H37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I37" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">열 단어를 다섯 단어로 줄이는 것은 재조합이 아니라 다른 방식의 표현 — 다음 레벨</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">열 단어 다섯 단어로 줄이면서 내용 손실이 없게 만드는 거는 진짜 그다음 레벨이에요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L37" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M37" s="11" t="str"/>
+      <x:c r="N37" s="11" t="str"/>
+      <x:c r="O37" s="11" t="str"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:45:16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:45:16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G38" s="11" t="str"/>
+      <x:c r="H38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I38" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">헤드라이닝을 딸깍으로 AI에게 시키는 순간 그 단계에 도달하지 못함</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">딸깍으로 AI한테 시켜서 해 보겠다라는 마음가짐으로 시켜 보잖아요. 거기서 이미 끝났어요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M38" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N38" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O38" s="11" t="str"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:52:05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:52:05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G39" s="11" t="str"/>
+      <x:c r="H39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I39" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">모든 문서는 히어로 섹션과 그 아래 섹션에서 승부가 남</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">섹션 1, 2에서 승부를 봐야지 지금 모든 단위의 모든 문서에서 그래요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M39" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N39" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O39" s="11" t="str"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">01:59:22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1:59:22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G40" s="11" t="str"/>
+      <x:c r="H40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I40" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">UX 결과물을 눈으로 확인하기 전에 랜딩 페이지로 넘어가지 말 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">그걸 안 보고 랜딩 페이지로도 넘어가지 말라는 거예요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M40" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N40" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O40" s="11" t="str"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">31:16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">31:16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G41" s="11" t="str"/>
+      <x:c r="H41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I41" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">오래 걸릴 작업은 작업 범위 선언을 확인하고 시작하는 습관</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">무슨 작업하든지 오래 걸릴 것 같은 작업은 이걸 확인하고 시작하는 습관을 꼭 들이세요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M41" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N41" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O41" s="11" t="str"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">32:43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">32:43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G42" s="11" t="str"/>
+      <x:c r="H42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I42" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">태스크는 상세해 보이지만 완전하지 않다</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">테스크는 상세해 보이지만 완전하지 않아요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M42" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MUST</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N42" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O42" s="11" t="str"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">33:37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">33:47</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CORE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I43" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">모르는 용어를 인지한 즉시 대응하는 것이 메타인지이고 생산성 차이를 만듦</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">내가 인지했을 때 그 인지 새롭게 내 스스로 진단한 상황에 대해서 아주 예민하게 즉시 대응하는 거죠. 메타인지죠</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L43" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M43" s="11" t="str"/>
+      <x:c r="N43" s="11" t="str"/>
+      <x:c r="O43" s="11" t="str"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">U16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미검토 세션</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">26일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3교시</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">45:52</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">45:47</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Y</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AVOID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I44" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">객관식 선택지라도 원하는 답이 아니면 절대 누르지 말고 말로 할 것</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">내가 원하는 피드백이 아닌 것은 절대 누르지 마세요</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L44" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">N</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M44" s="11" t="str"/>
+      <x:c r="N44" s="11" t="str"/>
+      <x:c r="O44" s="11" t="str"/>
+    </x:row>
+  </x:sheetData>
+</x:worksheet>
 </file>
</xml_diff>